<commit_message>
Add New York dental clinics data 2026-06-10
</commit_message>
<xml_diff>
--- a/output/New York_Dental_Clinics.xlsx
+++ b/output/New York_Dental_Clinics.xlsx
@@ -972,17 +972,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Midtown Dental Care Associates</t>
+          <t>New York Dental Office</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>(212) 685-4730</t>
+          <t>(212) 548-3261</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>12 E 41st St Ste 1100, New York, NY 10017, USA</t>
+          <t>245 E 63rd St #110, New York, NY 10065, USA</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -992,25 +992,25 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>https://www.midtowndentalcareassociates.com/?utm_source=gmb&amp;utm_medium=organic</t>
+          <t>https://www.newyorkdentaloffice.com/</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>573</v>
+        <v>469</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 7:00 PM</t>
+          <t>Monday: 8:30 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>40.752382</v>
+        <v>40.7633351</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>-73.980661</v>
+        <v>-73.9627181</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>100</v>
@@ -1027,17 +1027,17 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Expert Dental - Midtown</t>
+          <t>Midtown Dental Care Associates</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>(212) 763-3383</t>
+          <t>(212) 685-4730</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>110 E 40th St #104, New York, NY 10016, USA</t>
+          <t>12 E 41st St Ste 1100, New York, NY 10017, USA</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1047,25 +1047,25 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>https://www.expertdentalnyc.com/</t>
+          <t>https://www.midtowndentalcareassociates.com/?utm_source=gmb&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>4.5</v>
+        <v>4.9</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>2156</v>
+        <v>573</v>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 7:00 PM</t>
+          <t>Monday: 8:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J8" s="9" t="n">
-        <v>40.7503706</v>
+        <v>40.752382</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-73.9780354</v>
+        <v>-73.980661</v>
       </c>
       <c r="L8" s="9" t="n">
         <v>100</v>
@@ -1082,17 +1082,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>New York Dental Office</t>
+          <t>NYC Smile Spa</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>(212) 548-3261</t>
+          <t>(646) 374-2242</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>245 E 63rd St #110, New York, NY 10065, USA</t>
+          <t>30 E 60th St Ste 1201, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1102,25 +1102,25 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>https://www.newyorkdentaloffice.com/</t>
+          <t>https://www.nycsmilespa.com/</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>469</v>
+        <v>395</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:30 AM – 5:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>40.7633351</v>
+        <v>40.7637066</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>-73.9627181</v>
+        <v>-73.970242</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>100</v>
@@ -1137,17 +1137,17 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>NYC Dental Center</t>
+          <t>Studio Smiles NYC</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>(646) 861-3070</t>
+          <t>(646) 470-1376</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>216 E 39th St #1, New York, NY 10016, USA</t>
+          <t>41 Park Ave # 1C, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1157,28 +1157,28 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>https://weence.com/dentists/new-york-1/nyc-dental-center/</t>
+          <t>http://www.studiosmilesnyc.com/</t>
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>255</v>
+        <v>611</v>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J10" s="9" t="n">
-        <v>40.7483698</v>
+        <v>40.748366</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>-73.9752108</v>
+        <v>-73.97995039999999</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="M10" s="8" t="inlineStr">
         <is>
@@ -1192,17 +1192,17 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>NYC Smile Spa</t>
+          <t>212 Dental Care</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>(646) 374-2242</t>
+          <t>(888) 506-9583</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>30 E 60th St Ste 1201, New York, NY 10022, USA</t>
+          <t>286 Madison Ave 10th Floor, New York, NY 10017, USA</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1212,25 +1212,25 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>https://www.nycsmilespa.com/</t>
+          <t>http://212dentalcare.com/</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>395</v>
+        <v>3285</v>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 8:00 PM</t>
         </is>
       </c>
       <c r="J11" s="7" t="n">
-        <v>40.7637066</v>
+        <v>40.751693</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>-73.970242</v>
+        <v>-73.9803106</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>100</v>
@@ -1247,17 +1247,17 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Studio Smiles NYC</t>
+          <t>NYC Dental Center</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>(646) 470-1376</t>
+          <t>(646) 861-3070</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>41 Park Ave # 1C, New York, NY 10016, USA</t>
+          <t>216 E 39th St #1, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1267,28 +1267,28 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>http://www.studiosmilesnyc.com/</t>
+          <t>https://weence.com/dentists/new-york-1/nyc-dental-center/</t>
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>4.9</v>
+        <v>4.4</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>611</v>
+        <v>255</v>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 10:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J12" s="9" t="n">
-        <v>40.748366</v>
+        <v>40.7483698</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>-73.97995039999999</v>
+        <v>-73.9752108</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="M12" s="8" t="inlineStr">
         <is>
@@ -1302,17 +1302,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>212 Dental Care</t>
+          <t>Lumia Dental PLLC</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>(888) 506-9583</t>
+          <t>(212) 287-1275</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>286 Madison Ave 10th Floor, New York, NY 10017, USA</t>
+          <t>160 Broadway #1004, New York, NY 10038, USA</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1322,25 +1322,25 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>http://212dentalcare.com/</t>
+          <t>https://www.lumiadental.com/</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>3285</v>
+        <v>768</v>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 8:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>40.751693</v>
+        <v>40.70937199999999</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>-73.9803106</v>
+        <v>-74.00997500000001</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>100</v>
@@ -1357,17 +1357,17 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Lumia Dental PLLC</t>
+          <t>Expert Dental - Midtown</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>(212) 287-1275</t>
+          <t>(212) 763-3383</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>160 Broadway #1004, New York, NY 10038, USA</t>
+          <t>110 E 40th St #104, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1377,25 +1377,25 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>https://www.lumiadental.com/</t>
+          <t>https://www.expertdentalnyc.com/</t>
         </is>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>768</v>
+        <v>2156</v>
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 9:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>40.70937199999999</v>
+        <v>40.7503706</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>-74.00997500000001</v>
+        <v>-73.9780354</v>
       </c>
       <c r="L14" s="9" t="n">
         <v>100</v>
@@ -1412,17 +1412,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>172 NYC Dental</t>
+          <t>Midtown Dental Group Fashion District</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>(646) 921-5541</t>
+          <t>(212) 730-4440</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>172 Madison Ave Comm 1, New York, NY 10016, USA</t>
+          <t>241 W 37th St Ground Floor, New York, NY 10018, USA</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1432,25 +1432,25 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>https://172nycdental.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gmb</t>
+          <t>http://www.midtowndentalgroup.com/</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>260</v>
+        <v>734</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Monday: 7:30 AM – 6:30 PM</t>
+          <t>Monday: 9:00 AM – 5:45 PM</t>
         </is>
       </c>
       <c r="J15" s="7" t="n">
-        <v>40.7474307</v>
+        <v>40.7538706</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-73.9835995</v>
+        <v>-73.9909457</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>100</v>
@@ -1467,17 +1467,17 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Midtown Dental Group Fashion District</t>
+          <t>172 NYC Dental</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>(212) 730-4440</t>
+          <t>(646) 921-5541</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>241 W 37th St Ground Floor, New York, NY 10018, USA</t>
+          <t>172 Madison Ave Comm 1, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1487,25 +1487,25 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>http://www.midtowndentalgroup.com/</t>
+          <t>https://172nycdental.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gmb</t>
         </is>
       </c>
       <c r="G16" s="9" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>734</v>
+        <v>260</v>
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:45 PM</t>
+          <t>Monday: 7:30 AM – 6:30 PM</t>
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>40.7538706</v>
+        <v>40.7474307</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>-73.9909457</v>
+        <v>-73.9835995</v>
       </c>
       <c r="L16" s="9" t="n">
         <v>100</v>
@@ -1632,17 +1632,17 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Tribeca Dental Care</t>
+          <t>PDA Dental</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>(212) 431-4582</t>
+          <t>(212) 256-9583</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>402 Broadway, New York, NY 10013, USA</t>
+          <t>150 Broadway #1310, New York, NY 10038, USA</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1652,25 +1652,25 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>https://tribecanydentistoffice.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gbp</t>
+          <t>https://pdadental.com/</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>1153</v>
+        <v>730</v>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 6:30 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J19" s="7" t="n">
-        <v>40.7186949</v>
+        <v>40.7092051</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>-74.0021775</v>
+        <v>-74.01010840000001</v>
       </c>
       <c r="L19" s="7" t="n">
         <v>100</v>
@@ -1742,17 +1742,17 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Preferred Dental Care - Chelsea Dentist</t>
+          <t>Tribeca Dental Care</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>(212) 594-7171</t>
+          <t>(212) 431-4582</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>135 W 27th St, New York, NY 10001, USA</t>
+          <t>402 Broadway, New York, NY 10013, USA</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1762,25 +1762,25 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>https://www.preferreddentalcare.com/locations/chelsea-ny-location</t>
+          <t>https://tribecanydentistoffice.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gbp</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>2341</v>
+        <v>1153</v>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Monday: 7:00 AM – 9:00 PM</t>
+          <t>Monday: 10:00 AM – 6:30 PM</t>
         </is>
       </c>
       <c r="J21" s="7" t="n">
-        <v>40.7462879</v>
+        <v>40.7186949</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>-73.9924206</v>
+        <v>-74.0021775</v>
       </c>
       <c r="L21" s="7" t="n">
         <v>100</v>
@@ -1797,17 +1797,17 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>PDA Dental</t>
+          <t>New York Family Dental Arts</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>(212) 256-9583</t>
+          <t>(212) 628-3300</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>150 Broadway #1310, New York, NY 10038, USA</t>
+          <t>200 E 72nd St, New York, NY 10021, USA</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -1817,25 +1817,25 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>https://pdadental.com/</t>
+          <t>http://www.dentalartsny.com/</t>
         </is>
       </c>
       <c r="G22" s="9" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>730</v>
+        <v>571</v>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>40.7092051</v>
+        <v>40.7693746</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>-74.01010840000001</v>
+        <v>-73.9602924</v>
       </c>
       <c r="L22" s="9" t="n">
         <v>100</v>
@@ -1852,17 +1852,17 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>TriBeCa Dental Associates | Murray</t>
+          <t>Park Smiles NYC Cosmetic Dentistry</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>(212) 671-3749</t>
+          <t>(212) 988-6724</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>21 Murray St 4th floor, New York, NY 10007, USA</t>
+          <t>1175 Park Ave #1d, New York, NY 10128, USA</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -1872,25 +1872,25 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>https://tribeca.dental/</t>
+          <t>https://www.parksmilesnyc.com/our-locations/cargenie-hill-dentist/</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>1501</v>
+        <v>546</v>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 4:00 PM</t>
+          <t>Monday: 7:45 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J23" s="7" t="n">
-        <v>40.7137936</v>
+        <v>40.7843921</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>-74.0081888</v>
+        <v>-73.9538405</v>
       </c>
       <c r="L23" s="7" t="n">
         <v>100</v>
@@ -1907,17 +1907,17 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Park Smiles NYC Cosmetic Dentistry</t>
+          <t>TriBeCa Dental Associates | Murray</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>(212) 988-6724</t>
+          <t>(212) 671-3749</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>1175 Park Ave #1d, New York, NY 10128, USA</t>
+          <t>21 Murray St 4th floor, New York, NY 10007, USA</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -1927,25 +1927,25 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>https://www.parksmilesnyc.com/our-locations/cargenie-hill-dentist/</t>
+          <t>https://tribeca.dental/</t>
         </is>
       </c>
       <c r="G24" s="9" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>546</v>
+        <v>1501</v>
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Monday: 7:45 AM – 5:00 PM</t>
+          <t>Monday: 8:00 AM – 4:00 PM</t>
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>40.7843921</v>
+        <v>40.7137936</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>-73.9538405</v>
+        <v>-74.0081888</v>
       </c>
       <c r="L24" s="9" t="n">
         <v>100</v>
@@ -1962,17 +1962,17 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Sachar Dental NYC</t>
+          <t>New York General Dentistry</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>(212) 752-1163</t>
+          <t>(212) 838-0842</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>20 E 46th St Rm 1301, New York, NY 10017, USA</t>
+          <t>133 E 58th St Ste 409, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1982,25 +1982,25 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>https://www.sachardental.com/</t>
+          <t>https://newyorkgeneraldentistry.com/?utm_source=GMBlisting&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>414</v>
+        <v>371</v>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 8:30 AM – 5:30 PM</t>
         </is>
       </c>
       <c r="J25" s="7" t="n">
-        <v>40.7554749</v>
+        <v>40.7619525</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>-73.9779336</v>
+        <v>-73.9689326</v>
       </c>
       <c r="L25" s="7" t="n">
         <v>100</v>
@@ -2017,17 +2017,17 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>New York General Dentistry</t>
+          <t>Sachar Dental NYC</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>(212) 838-0842</t>
+          <t>(212) 752-1163</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>133 E 58th St Ste 409, New York, NY 10022, USA</t>
+          <t>20 E 46th St Rm 1301, New York, NY 10017, USA</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -2037,25 +2037,25 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>https://newyorkgeneraldentistry.com/?utm_source=GMBlisting&amp;utm_medium=organic</t>
+          <t>https://www.sachardental.com/</t>
         </is>
       </c>
       <c r="G26" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>371</v>
+        <v>414</v>
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:30 AM – 5:30 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J26" s="9" t="n">
-        <v>40.7619525</v>
+        <v>40.7554749</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>-73.9689326</v>
+        <v>-73.9779336</v>
       </c>
       <c r="L26" s="9" t="n">
         <v>100</v>
@@ -2127,17 +2127,17 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>The Exchange Dental Group</t>
+          <t>My NYC Dentist - Hudson Street Dental</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>(646) 780-5410</t>
+          <t>(212) 359-0064</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>39 Broadway Rm 2115, New York, NY 10006, USA</t>
+          <t>90 Vandam St, New York, NY 10013, USA</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2147,25 +2147,25 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>https://www.theexchangedentalgroup.com/</t>
+          <t>https://www.mynyc-dentist.com/</t>
         </is>
       </c>
       <c r="G28" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>1249</v>
+        <v>289</v>
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 7:00 PM</t>
+          <t>Monday: 8:30 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J28" s="9" t="n">
-        <v>40.7063221</v>
+        <v>40.7265687</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>-74.01333289999999</v>
+        <v>-74.00812239999999</v>
       </c>
       <c r="L28" s="9" t="n">
         <v>100</v>
@@ -2182,17 +2182,17 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Manhattan Dental Spa: John Vargas DDS, Allison Gordon DMD, &amp; Mitchell Charnas DMD</t>
+          <t>The Exchange Dental Group</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>(212) 683-2530</t>
+          <t>(646) 780-5410</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>200 Madison Ave Ste 2201, New York, NY 10016, USA</t>
+          <t>39 Broadway Rm 2115, New York, NY 10006, USA</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2202,25 +2202,25 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>https://manhattandentalspa.com/?utm_source=gmb&amp;utm_medium=organic</t>
+          <t>https://www.theexchangedentalgroup.com/</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>728</v>
+        <v>1249</v>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 7:00 PM</t>
+          <t>Monday: 8:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>40.7486953</v>
+        <v>40.7063221</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>-73.98253629999999</v>
+        <v>-74.01333289999999</v>
       </c>
       <c r="L29" s="7" t="n">
         <v>100</v>
@@ -2237,17 +2237,17 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Smile Arts of NY</t>
+          <t>Manhattan Dental Spa: John Vargas DDS, Allison Gordon DMD, &amp; Mitchell Charnas DMD</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>(212) 537-6923</t>
+          <t>(212) 683-2530</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>30 E 40th St #105, New York, NY 10016, USA</t>
+          <t>200 Madison Ave Ste 2201, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -2257,25 +2257,25 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>http://www.smileartsofny.com/</t>
+          <t>https://manhattandentalspa.com/?utm_source=gmb&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G30" s="9" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>797</v>
+        <v>728</v>
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 7:30 PM</t>
+          <t>Monday: 9:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J30" s="9" t="n">
-        <v>40.751178</v>
+        <v>40.7486953</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>-73.97962799999999</v>
+        <v>-73.98253629999999</v>
       </c>
       <c r="L30" s="9" t="n">
         <v>100</v>
@@ -2292,17 +2292,17 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>SoHo Dental Group NYC</t>
+          <t>Wall Street Dental Spa - Financial District</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>(212) 878-7646</t>
+          <t>(212) 514-5514</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>552 Broadway #505, New York, NY 10012, USA</t>
+          <t>30 Wall St #720, New York, NY 10005, USA</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2312,14 +2312,14 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>https://www.sohodentalgroup.com/?utm_campaign=gmb&amp;utm_medium=organic&amp;utm_source=gmb</t>
+          <t>https://wallstdentalspanyc.com/</t>
         </is>
       </c>
       <c r="G31" s="7" t="n">
         <v>4.8</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>540</v>
+        <v>1406</v>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
@@ -2327,10 +2327,10 @@
         </is>
       </c>
       <c r="J31" s="7" t="n">
-        <v>40.7237243</v>
+        <v>40.7069897</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>-73.99803159999999</v>
+        <v>-74.01027259999999</v>
       </c>
       <c r="L31" s="7" t="n">
         <v>100</v>
@@ -2347,17 +2347,17 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Diamond District Dental NYC - Midtown Dentist</t>
+          <t>SoHo Dental Group NYC</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>(212) 759-5595</t>
+          <t>(212) 878-7646</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>10 W 46th St #1401, New York, NY 10036, USA</t>
+          <t>552 Broadway #505, New York, NY 10012, USA</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -2367,14 +2367,14 @@
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>https://www.dddentalnyc.com/?utm_campaign=gmb</t>
+          <t>https://www.sohodentalgroup.com/?utm_campaign=gmb&amp;utm_medium=organic&amp;utm_source=gmb</t>
         </is>
       </c>
       <c r="G32" s="9" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>595</v>
+        <v>540</v>
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
@@ -2382,10 +2382,10 @@
         </is>
       </c>
       <c r="J32" s="9" t="n">
-        <v>40.7563177</v>
+        <v>40.7237243</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>-73.9800044</v>
+        <v>-73.99803159999999</v>
       </c>
       <c r="L32" s="9" t="n">
         <v>100</v>
@@ -2402,17 +2402,17 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Manhattan Bridge Orthodontics</t>
+          <t>Diamond District Dental NYC - Midtown Dentist</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>(212) 274-0477</t>
+          <t>(212) 759-5595</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>77 Bowery 6th Floor, New York, NY 10002, USA</t>
+          <t>10 W 46th St #1401, New York, NY 10036, USA</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2422,25 +2422,25 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>https://www.manhattanbridgeortho.com/</t>
+          <t>https://www.dddentalnyc.com/?utm_campaign=gmb</t>
         </is>
       </c>
       <c r="G33" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>1514</v>
+        <v>595</v>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 7:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>40.71666949999999</v>
+        <v>40.7563177</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>-73.99553539999999</v>
+        <v>-73.9800044</v>
       </c>
       <c r="L33" s="7" t="n">
         <v>100</v>
@@ -2457,17 +2457,17 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>iSmile Orthodontics - NYC</t>
+          <t>Manhattan Bridge Orthodontics</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>(646) 863-2181</t>
+          <t>(212) 274-0477</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>4779 Broadway, New York, NY 10034, USA</t>
+          <t>77 Bowery 6th Floor, New York, NY 10002, USA</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
@@ -2477,25 +2477,25 @@
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>https://ismileorthodontics.com/inwood/</t>
+          <t>https://www.manhattanbridgeortho.com/</t>
         </is>
       </c>
       <c r="G34" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>1006</v>
+        <v>1514</v>
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 10:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J34" s="9" t="n">
-        <v>40.8659992</v>
+        <v>40.71666949999999</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>-73.92655979999999</v>
+        <v>-73.99553539999999</v>
       </c>
       <c r="L34" s="9" t="n">
         <v>100</v>
@@ -2567,17 +2567,17 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Manhattan EastSide Orthodontics</t>
+          <t>iSmile Orthodontics - NYC</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>(212) 289-8989</t>
+          <t>(646) 863-2181</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>207 E 94th St #501, New York, NY 10128, USA</t>
+          <t>4779 Broadway, New York, NY 10034, USA</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -2587,25 +2587,25 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>https://manhattaneastsideorthodontics.com/</t>
+          <t>https://ismileorthodontics.com/inwood/</t>
         </is>
       </c>
       <c r="G36" s="9" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>429</v>
+        <v>1006</v>
       </c>
       <c r="I36" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J36" s="9" t="n">
-        <v>40.783778</v>
+        <v>40.8659992</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>-73.949438</v>
+        <v>-73.92655979999999</v>
       </c>
       <c r="L36" s="9" t="n">
         <v>100</v>
@@ -2622,17 +2622,17 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Bronsky Orthodontics</t>
+          <t>Manhattan EastSide Orthodontics</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>(212) 758-0040</t>
+          <t>(212) 289-8989</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>530 Park Ave APT 1G, New York, NY 10065, USA</t>
+          <t>207 E 94th St #501, New York, NY 10128, USA</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -2642,25 +2642,25 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>http://www.bronskyorthodontics.com/?utm_source=GMBlisting&amp;utm_medium=organic</t>
+          <t>https://manhattaneastsideorthodontics.com/</t>
         </is>
       </c>
       <c r="G37" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>481</v>
+        <v>429</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 5:00 PM</t>
+          <t>Monday: 9:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J37" s="7" t="n">
-        <v>40.7641462</v>
+        <v>40.783778</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>-73.96946849999999</v>
+        <v>-73.949438</v>
       </c>
       <c r="L37" s="7" t="n">
         <v>100</v>
@@ -2677,17 +2677,17 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Smile Pop - Dr. Courtney Barry Orthodontist</t>
+          <t>Bronsky Orthodontics</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>(646) 770-2091</t>
+          <t>(212) 758-0040</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>76 Madison Ave, New York, NY 10016, USA</t>
+          <t>530 Park Ave APT 1G, New York, NY 10065, USA</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -2697,25 +2697,25 @@
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>http://www.smilepop.com/</t>
+          <t>http://www.bronskyorthodontics.com/?utm_source=GMBlisting&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G38" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>444</v>
+        <v>481</v>
       </c>
       <c r="I38" s="9" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 4:00 PM</t>
+          <t>Monday: 8:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J38" s="9" t="n">
-        <v>40.74397099999999</v>
+        <v>40.7641462</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>-73.9860561</v>
+        <v>-73.96946849999999</v>
       </c>
       <c r="L38" s="9" t="n">
         <v>100</v>
@@ -2732,17 +2732,17 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Brite Orthodontics - Harlem (Central Park North Orthodontics)</t>
+          <t>Smile Pop - Dr. Courtney Barry Orthodontist</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>(212) 866-9800</t>
+          <t>(646) 770-2091</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>1851 Adam Clayton Powell Jr Blvd, New York, NY 10026, USA</t>
+          <t>76 Madison Ave, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2752,25 +2752,25 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>https://www.briteorthodontics.com/locations/newyork-ny/</t>
+          <t>http://www.smilepop.com/</t>
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>673</v>
+        <v>444</v>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: 10:00 AM – 4:00 PM</t>
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>40.8009348</v>
+        <v>40.74397099999999</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>-73.95373900000001</v>
+        <v>-73.9860561</v>
       </c>
       <c r="L39" s="7" t="n">
         <v>100</v>
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Goodman Orthodontics</t>
+          <t>Brite Orthodontics - Harlem (Central Park North Orthodontics)</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>(212) 688-4663</t>
+          <t>(212) 866-9800</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>440 E 57th St B, New York, NY 10022, USA</t>
+          <t>1851 Adam Clayton Powell Jr Blvd, New York, NY 10026, USA</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2862,25 +2862,25 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>http://www.goodortho.com/</t>
+          <t>https://www.briteorthodontics.com/locations/newyork-ny/</t>
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>275</v>
+        <v>673</v>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 4:00 PM</t>
+          <t>Monday: 9:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>40.7575229</v>
+        <v>40.8009348</v>
       </c>
       <c r="K41" s="7" t="n">
-        <v>-73.9616418</v>
+        <v>-73.95373900000001</v>
       </c>
       <c r="L41" s="7" t="n">
         <v>100</v>
@@ -2897,17 +2897,17 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Gramercy Orthodontics</t>
+          <t>Goodman Orthodontics</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>(212) 777-9177</t>
+          <t>(212) 688-4663</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>200 E 15th St STE PRB, New York, NY 10003, USA</t>
+          <t>440 E 57th St B, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
@@ -2917,28 +2917,28 @@
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>https://gramercyorthonyc.com/</t>
+          <t>http://www.goodortho.com/</t>
         </is>
       </c>
       <c r="G42" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>161</v>
+        <v>275</v>
       </c>
       <c r="I42" s="9" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 7:00 PM</t>
+          <t>Monday: 8:00 AM – 4:00 PM</t>
         </is>
       </c>
       <c r="J42" s="9" t="n">
-        <v>40.7337844</v>
+        <v>40.7575229</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>-73.98647919999999</v>
+        <v>-73.9616418</v>
       </c>
       <c r="L42" s="9" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
@@ -2952,17 +2952,17 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>House of Orthodontia - Manhattan</t>
+          <t>Gramercy Orthodontics</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>(212) 392-4789</t>
+          <t>(212) 777-9177</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>601 E 12th St, New York, NY 10009, USA</t>
+          <t>200 E 15th St STE PRB, New York, NY 10003, USA</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -2972,25 +2972,25 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>https://houseoforthodontia.com/</t>
+          <t>https://gramercyorthonyc.com/</t>
         </is>
       </c>
       <c r="G43" s="7" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>101</v>
+        <v>161</v>
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>Monday: Closed</t>
+          <t>Monday: 10:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J43" s="7" t="n">
-        <v>40.7281888</v>
+        <v>40.7337844</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>-73.9788071</v>
+        <v>-73.98647919999999</v>
       </c>
       <c r="L43" s="7" t="n">
         <v>93</v>
@@ -3007,17 +3007,17 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Manhattan Family Orthodontics-Uptown</t>
+          <t>House of Orthodontia - Manhattan</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>(347) 767-5668</t>
+          <t>(212) 392-4789</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>207 E 63rd St, New York, NY 10022, USA</t>
+          <t>601 E 12th St, New York, NY 10009, USA</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -3027,25 +3027,25 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>https://www.manhattanfamilyorthodontics.com/</t>
+          <t>https://houseoforthodontia.com/</t>
         </is>
       </c>
       <c r="G44" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>159</v>
+        <v>101</v>
       </c>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>Monday: 1:00 – 6:00 PM</t>
+          <t>Monday: Closed</t>
         </is>
       </c>
       <c r="J44" s="9" t="n">
-        <v>40.7640232</v>
+        <v>40.7281888</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>-73.96417579999999</v>
+        <v>-73.9788071</v>
       </c>
       <c r="L44" s="9" t="n">
         <v>93</v>
@@ -3062,34 +3062,34 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Jackson Heights Orthodontics</t>
+          <t>Gibbs Orthodontic Associates, P.C : Invisalign, Braces and Dentofacial Orthopedics</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>(718) 335-4444</t>
+          <t>(212) 535-4111</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>37-43 77th St, Jackson Heights, NY 11372, USA</t>
+          <t>40 E 84th St, New York, NY 10028, USA</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>Jackson Heights</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>http://jhoortho.com/</t>
+          <t>https://www.gibbsortho.com/</t>
         </is>
       </c>
       <c r="G45" s="7" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>1337</v>
+        <v>186</v>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
@@ -3097,13 +3097,13 @@
         </is>
       </c>
       <c r="J45" s="7" t="n">
-        <v>40.7479692</v>
+        <v>40.7793093</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>-73.88860989999999</v>
+        <v>-73.95947029999999</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
@@ -3227,17 +3227,17 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Bronsky Orthodontics - Tribeca</t>
+          <t>Manhattan Family Orthodontics-Uptown</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>(212) 758-0040</t>
+          <t>(347) 767-5668</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>15 Harrison St Ground Floor, New York, NY 10013, USA</t>
+          <t>207 E 63rd St, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -3247,28 +3247,28 @@
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>http://www.bronskyorthodontics.com/?UTM_source=GBP_Listing&amp;UTM_medium=Organic</t>
+          <t>https://www.manhattanfamilyorthodontics.com/</t>
         </is>
       </c>
       <c r="G48" s="9" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>271</v>
+        <v>159</v>
       </c>
       <c r="I48" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 5:00 PM</t>
+          <t>Monday: 1:00 – 6:00 PM</t>
         </is>
       </c>
       <c r="J48" s="9" t="n">
-        <v>40.7185619</v>
+        <v>40.7640232</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>-74.0098603</v>
+        <v>-73.96417579999999</v>
       </c>
       <c r="L48" s="9" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M48" s="8" t="inlineStr">
         <is>
@@ -3282,17 +3282,17 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Upper Eastside Orthodontists</t>
+          <t>Salzer Orthodontics, Dr. Jennifer Salzer</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>(212) 360-0835</t>
+          <t>(212) 755-2333</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>153 E 87th St APT 1B, New York, NY 10128, USA</t>
+          <t>553 Park Ave, New York, NY 10065, USA</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -3302,28 +3302,28 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>https://www.ueso.org/?utm_source=local_directory&amp;utm_medium=referral&amp;utm_campaign=directory-listing</t>
+          <t>https://lsortho.com/contact-orthodontist-nyc</t>
         </is>
       </c>
       <c r="G49" s="7" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>476</v>
+        <v>177</v>
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>Monday: Closed</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J49" s="7" t="n">
-        <v>40.7802182</v>
+        <v>40.7645406</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>-73.9546495</v>
+        <v>-73.9683215</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M49" s="8" t="inlineStr">
         <is>
@@ -3392,17 +3392,17 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Salzer Orthodontics, Dr. Jennifer Salzer</t>
+          <t>Bronsky Orthodontics - Tribeca</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>(212) 755-2333</t>
+          <t>(212) 758-0040</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>553 Park Ave, New York, NY 10065, USA</t>
+          <t>15 Harrison St Ground Floor, New York, NY 10013, USA</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -3412,28 +3412,28 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>https://lsortho.com/contact-orthodontist-nyc</t>
+          <t>http://www.bronskyorthodontics.com/?UTM_source=GBP_Listing&amp;UTM_medium=Organic</t>
         </is>
       </c>
       <c r="G51" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>177</v>
+        <v>271</v>
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J51" s="7" t="n">
-        <v>40.7645406</v>
+        <v>40.7185619</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>-73.9683215</v>
+        <v>-74.0098603</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M51" s="8" t="inlineStr">
         <is>
@@ -3447,17 +3447,17 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Mid-Manhattan Oral Surgery, PC</t>
+          <t>Upper Eastside Orthodontists</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>(212) 918-1859</t>
+          <t>(212) 360-0835</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>36 West 44th Street, Suite 600 Between, 5th and 6th Avenue, New York, NY 10036, USA</t>
+          <t>153 E 87th St APT 1B, New York, NY 10128, USA</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -3467,25 +3467,25 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>https://www.midmanhattanoralsurgery.com/</t>
+          <t>https://www.ueso.org/?utm_source=local_directory&amp;utm_medium=referral&amp;utm_campaign=directory-listing</t>
         </is>
       </c>
       <c r="G52" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>895</v>
+        <v>476</v>
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 5:00 PM</t>
+          <t>Monday: Closed</t>
         </is>
       </c>
       <c r="J52" s="9" t="n">
-        <v>40.7555517</v>
+        <v>40.7802182</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>-73.9819631</v>
+        <v>-73.9546495</v>
       </c>
       <c r="L52" s="9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add scrape results 2026-06-15
</commit_message>
<xml_diff>
--- a/output/New York_Dental_Clinics.xlsx
+++ b/output/New York_Dental_Clinics.xlsx
@@ -599,10 +599,10 @@
         <v>50</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>0</v>
@@ -628,10 +628,10 @@
         <v>50</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>0</v>
@@ -779,7 +779,7 @@
         <v>4.9</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1830</v>
+        <v>1835</v>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
@@ -807,17 +807,17 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>New York University College of Dentistry</t>
+          <t>Sky Dental</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>(212) 998-9800</t>
+          <t>(212) 600-1996</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>345 E 24th St, New York, NY 10010, USA</t>
+          <t>111 Broadway Suite 1304, New York, NY 10006, USA</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -827,32 +827,32 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>http://dental.nyu.edu/</t>
+          <t>https://skydentalnyc.com/?utm_campaign=gmb</t>
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>3.6</v>
+        <v>4.9</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>1228</v>
+        <v>2658</v>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 8:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J4" s="9" t="n">
-        <v>40.7378213</v>
+        <v>40.7086853</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>-73.97840579999999</v>
+        <v>-74.01154869999999</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>63</v>
-      </c>
-      <c r="M4" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>100</v>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -862,17 +862,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Sky Dental</t>
+          <t>Pearl Dental NYC</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>(212) 600-1996</t>
+          <t>(212) 344-9317</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>111 Broadway Suite 1304, New York, NY 10006, USA</t>
+          <t>233 Broadway 18 Suite 1801, New York, NY 10279, USA</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -882,25 +882,25 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>https://skydentalnyc.com/?utm_campaign=gmb</t>
+          <t>https://www.pearldentalnyc.com/</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>2654</v>
+        <v>475</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>40.7086853</v>
+        <v>40.7123834</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-74.01154869999999</v>
+        <v>-74.0079386</v>
       </c>
       <c r="L5" s="7" t="n">
         <v>100</v>
@@ -917,17 +917,17 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>ORAL Dental Studio NYC</t>
+          <t>Midtown Dental Group Fashion District</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>(646) 663-7633</t>
+          <t>(212) 730-4440</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>131 Essex St Fl 2, New York, NY 10002, USA</t>
+          <t>241 W 37th St Ground Floor, New York, NY 10018, USA</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -937,25 +937,25 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>https://www.oraldentalstudio.com/</t>
+          <t>http://www.midtowndentalgroup.com/</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>458</v>
+        <v>737</v>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 9:00 AM – 5:45 PM</t>
         </is>
       </c>
       <c r="J6" s="9" t="n">
-        <v>40.7200496</v>
+        <v>40.7538706</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>-73.98762359999999</v>
+        <v>-73.9909457</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>100</v>
@@ -972,17 +972,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Expert Dental - Midtown</t>
+          <t>New York University College of Dentistry</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>(212) 763-3383</t>
+          <t>(212) 998-9800</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>110 E 40th St #104, New York, NY 10016, USA</t>
+          <t>345 E 24th St, New York, NY 10010, USA</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -992,32 +992,32 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>https://www.expertdentalnyc.com/</t>
+          <t>http://dental.nyu.edu/</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>2156</v>
+        <v>1227</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 7:00 PM</t>
+          <t>Monday: 8:00 AM – 8:00 PM</t>
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>40.7503706</v>
+        <v>40.7378213</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>-73.9780354</v>
+        <v>-73.97840579999999</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="M7" s="8" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>63</v>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1027,17 +1027,17 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>New York Dental Office</t>
+          <t>ORAL Dental Studio NYC</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>(212) 548-3261</t>
+          <t>(646) 663-7633</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>245 E 63rd St #110, New York, NY 10065, USA</t>
+          <t>131 Essex St Fl 2, New York, NY 10002, USA</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1047,25 +1047,25 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>https://www.newyorkdentaloffice.com/</t>
+          <t>https://www.oraldentalstudio.com/</t>
         </is>
       </c>
       <c r="G8" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>469</v>
+        <v>460</v>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:30 AM – 5:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J8" s="9" t="n">
-        <v>40.7633351</v>
+        <v>40.7200496</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-73.9627181</v>
+        <v>-73.98762359999999</v>
       </c>
       <c r="L8" s="9" t="n">
         <v>100</v>
@@ -1082,17 +1082,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Pearl Dental NYC</t>
+          <t>New York Dental Office</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>(212) 344-9317</t>
+          <t>(212) 548-3261</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>233 Broadway 18 Suite 1801, New York, NY 10279, USA</t>
+          <t>245 E 63rd St #110, New York, NY 10065, USA</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1102,25 +1102,25 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>https://www.pearldentalnyc.com/</t>
+          <t>https://www.newyorkdentaloffice.com/</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 5:00 PM</t>
+          <t>Monday: 8:30 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>40.7123834</v>
+        <v>40.7633351</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>-74.0079386</v>
+        <v>-73.9627181</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>100</v>
@@ -1137,17 +1137,17 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Midtown Dental Care Associates</t>
+          <t>Expert Dental - Midtown</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>(212) 685-4730</t>
+          <t>(212) 763-3383</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>12 E 41st St Ste 1100, New York, NY 10017, USA</t>
+          <t>110 E 40th St #104, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1157,25 +1157,25 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>https://www.midtowndentalcareassociates.com/?utm_source=gmb&amp;utm_medium=organic</t>
+          <t>https://www.expertdentalnyc.com/</t>
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>573</v>
+        <v>2159</v>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 7:00 PM</t>
+          <t>Monday: 9:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J10" s="9" t="n">
-        <v>40.752382</v>
+        <v>40.7503706</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>-73.980661</v>
+        <v>-73.9780354</v>
       </c>
       <c r="L10" s="9" t="n">
         <v>100</v>
@@ -1247,17 +1247,17 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>NYC Smile Spa</t>
+          <t>Midtown Dental Care Associates</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>(646) 374-2242</t>
+          <t>(212) 685-4730</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>30 E 60th St Ste 1201, New York, NY 10022, USA</t>
+          <t>12 E 41st St Ste 1100, New York, NY 10017, USA</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1267,25 +1267,25 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>https://www.nycsmilespa.com/</t>
+          <t>https://www.midtowndentalcareassociates.com/?utm_source=gmb&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G12" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>395</v>
+        <v>574</v>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J12" s="9" t="n">
-        <v>40.7637066</v>
+        <v>40.752382</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>-73.970242</v>
+        <v>-73.980661</v>
       </c>
       <c r="L12" s="9" t="n">
         <v>100</v>
@@ -1302,17 +1302,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>212 Dental Care</t>
+          <t>Diamond District Dental NYC - Midtown Dentist</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>(888) 506-9583</t>
+          <t>(212) 759-5595</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>286 Madison Ave 10th Floor, New York, NY 10017, USA</t>
+          <t>10 W 46th St #1401, New York, NY 10036, USA</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1322,25 +1322,25 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>http://212dentalcare.com/</t>
+          <t>https://www.dddentalnyc.com/?utm_campaign=gmb</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>3285</v>
+        <v>595</v>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 8:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>40.751693</v>
+        <v>40.7563177</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>-73.9803106</v>
+        <v>-73.9800044</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>100</v>
@@ -1357,17 +1357,17 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>SoHo Dental Group NYC</t>
+          <t>Studio Smiles NYC</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>(212) 878-7646</t>
+          <t>(646) 470-1376</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>552 Broadway #505, New York, NY 10012, USA</t>
+          <t>41 Park Ave # 1C, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1377,25 +1377,25 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>https://www.sohodentalgroup.com/?utm_campaign=gmb&amp;utm_medium=organic&amp;utm_source=gmb</t>
+          <t>http://www.studiosmilesnyc.com/</t>
         </is>
       </c>
       <c r="G14" s="9" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>540</v>
+        <v>610</v>
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>40.7237243</v>
+        <v>40.748366</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>-73.99803159999999</v>
+        <v>-73.97995039999999</v>
       </c>
       <c r="L14" s="9" t="n">
         <v>100</v>
@@ -1412,17 +1412,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Studio Smiles NYC</t>
+          <t>Lumia Dental PLLC</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>(646) 470-1376</t>
+          <t>(212) 287-1275</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>41 Park Ave # 1C, New York, NY 10016, USA</t>
+          <t>160 Broadway #1004, New York, NY 10038, USA</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1432,14 +1432,14 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>http://www.studiosmilesnyc.com/</t>
+          <t>https://www.lumiadental.com/</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>611</v>
+        <v>768</v>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
@@ -1447,10 +1447,10 @@
         </is>
       </c>
       <c r="J15" s="7" t="n">
-        <v>40.748366</v>
+        <v>40.70937199999999</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-73.97995039999999</v>
+        <v>-74.00997500000001</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>100</v>
@@ -1467,17 +1467,17 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Lumia Dental PLLC</t>
+          <t>My NYC Dentist - Hudson Street Dental</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>(212) 287-1275</t>
+          <t>(212) 359-0064</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>160 Broadway #1004, New York, NY 10038, USA</t>
+          <t>90 Vandam St, New York, NY 10013, USA</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1487,25 +1487,25 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>https://www.lumiadental.com/</t>
+          <t>https://www.mynyc-dentist.com/</t>
         </is>
       </c>
       <c r="G16" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>768</v>
+        <v>290</v>
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 6:00 PM</t>
+          <t>Monday: 8:30 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>40.70937199999999</v>
+        <v>40.7265687</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>-74.00997500000001</v>
+        <v>-74.00812239999999</v>
       </c>
       <c r="L16" s="9" t="n">
         <v>100</v>
@@ -1522,17 +1522,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>My NYC Dentist - Hudson Street Dental</t>
+          <t>SoHo Dental Group NYC</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>(212) 359-0064</t>
+          <t>(212) 878-7646</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>90 Vandam St, New York, NY 10013, USA</t>
+          <t>552 Broadway #505, New York, NY 10012, USA</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -1542,25 +1542,25 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>https://www.mynyc-dentist.com/</t>
+          <t>https://www.sohodentalgroup.com/?utm_campaign=gmb&amp;utm_medium=organic&amp;utm_source=gmb</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>289</v>
+        <v>540</v>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:30 AM – 6:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J17" s="7" t="n">
-        <v>40.7265687</v>
+        <v>40.7237243</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>-74.00812239999999</v>
+        <v>-73.99803159999999</v>
       </c>
       <c r="L17" s="7" t="n">
         <v>100</v>
@@ -1577,17 +1577,17 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Diamond District Dental NYC - Midtown Dentist</t>
+          <t>PDA Dental</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>(212) 759-5595</t>
+          <t>(212) 256-9583</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>10 W 46th St #1401, New York, NY 10036, USA</t>
+          <t>150 Broadway #1310, New York, NY 10038, USA</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1597,25 +1597,25 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>https://www.dddentalnyc.com/?utm_campaign=gmb</t>
+          <t>https://pdadental.com/</t>
         </is>
       </c>
       <c r="G18" s="9" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>595</v>
+        <v>730</v>
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>40.7563177</v>
+        <v>40.7092051</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>-73.9800044</v>
+        <v>-74.01010840000001</v>
       </c>
       <c r="L18" s="9" t="n">
         <v>100</v>
@@ -1632,17 +1632,17 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>City Dental Group NYC</t>
+          <t>The Exchange Dental Group</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>(212) 425-0505</t>
+          <t>(646) 780-5410</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>11 Broadway Lobby 4, New York, NY 10004, USA</t>
+          <t>39 Broadway Suite 2115, New York, NY 10006, USA</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1652,25 +1652,25 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>https://citydentalnyc.com/?utm_source=gbp&amp;utm_medium=organic&amp;utm_campaign=gbp-listing</t>
+          <t>https://www.theexchangedentalgroup.com/</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>311</v>
+        <v>1252</v>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:30 AM – 5:30 PM</t>
+          <t>Monday: 8:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J19" s="7" t="n">
-        <v>40.7053407</v>
+        <v>40.7063221</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>-74.01385759999999</v>
+        <v>-74.01333289999999</v>
       </c>
       <c r="L19" s="7" t="n">
         <v>100</v>
@@ -1687,17 +1687,17 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Wall Street Dental Spa - Financial District</t>
+          <t>Esthetix Dentist, NYC's Dental Implant &amp; Cosmetic Specialist</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>(212) 514-5514</t>
+          <t>(212) 795-9675</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>30 Wall St #720, New York, NY 10005, USA</t>
+          <t>285 Fort Washington Ave, New York, NY 10032, USA</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1707,25 +1707,25 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>https://wallstdentalspanyc.com/</t>
+          <t>https://www.esthetixdentalspa.com/</t>
         </is>
       </c>
       <c r="G20" s="9" t="n">
         <v>4.8</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>1406</v>
+        <v>1188</v>
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 8:00 PM</t>
         </is>
       </c>
       <c r="J20" s="9" t="n">
-        <v>40.7069897</v>
+        <v>40.8450168</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>-74.01027259999999</v>
+        <v>-73.9408416</v>
       </c>
       <c r="L20" s="9" t="n">
         <v>100</v>
@@ -1742,17 +1742,17 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Smile Cafe Dental Spa</t>
+          <t>Manhattan Dental Spa: John Vargas DDS, Allison Gordon DMD, &amp; Mitchell Charnas DMD</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>(212) 779-7743</t>
+          <t>(212) 683-2530</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Smile Cafe Dental Spa, 45 Park Ave Professional Unit 1, New York, NY 10016, USA</t>
+          <t>200 Madison Ave Ste 2201, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1762,25 +1762,25 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>http://www.smilecafeny.com/</t>
+          <t>https://manhattandentalspa.com/?utm_source=gmb&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>1099</v>
+        <v>729</v>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 8:00 PM</t>
+          <t>Monday: 9:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J21" s="7" t="n">
-        <v>40.7486592</v>
+        <v>40.7486953</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>-73.9797464</v>
+        <v>-73.98253629999999</v>
       </c>
       <c r="L21" s="7" t="n">
         <v>100</v>
@@ -1797,17 +1797,17 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>172 NYC Dental</t>
+          <t>NYC Dental of Upper East Side</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>(646) 921-5541</t>
+          <t>(212) 348-5492</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>172 Madison Ave Comm 1, New York, NY 10016, USA</t>
+          <t>1317 3rd Ave 2nd Floor, New York, NY 10021, USA</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -1817,28 +1817,28 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>https://172nycdental.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gmb</t>
+          <t>https://nycdent.com/</t>
         </is>
       </c>
       <c r="G22" s="9" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>260</v>
+        <v>305</v>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Monday: 7:30 AM – 6:30 PM</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>40.7474307</v>
+        <v>40.7718654</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>-73.9835995</v>
+        <v>-73.9586489</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="M22" s="8" t="inlineStr">
         <is>
@@ -1907,17 +1907,17 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>TriBeCa Dental Associates | Murray</t>
+          <t>Smile Design Manhattan</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>(212) 671-3749</t>
+          <t>(646) 278-4579</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>21 Murray St 4th floor, New York, NY 10007, USA</t>
+          <t>575 Madison Ave 23rd Floor, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -1927,25 +1927,25 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>https://tribeca.dental/</t>
+          <t>https://www.smiledesignmanhattan.com/?utm_source=gmb_auth</t>
         </is>
       </c>
       <c r="G24" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>1503</v>
+        <v>562</v>
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 4:00 PM</t>
+          <t>Monday: 9:00 AM – 8:00 PM</t>
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>40.7137936</v>
+        <v>40.761781</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>-74.0081888</v>
+        <v>-73.9723693</v>
       </c>
       <c r="L24" s="9" t="n">
         <v>100</v>
@@ -1962,17 +1962,17 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Park Smiles NYC Cosmetic Dentistry</t>
+          <t>Sachar Dental NYC</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>(212) 988-6724</t>
+          <t>(212) 752-1163</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>1175 Park Ave #1d, New York, NY 10128, USA</t>
+          <t>20 E 46th St Rm 1301, New York, NY 10017, USA</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1982,25 +1982,25 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>https://www.parksmilesnyc.com/our-locations/cargenie-hill-dentist/</t>
+          <t>https://www.sachardental.com/</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>546</v>
+        <v>415</v>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>Monday: 7:45 AM – 5:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J25" s="7" t="n">
-        <v>40.7843921</v>
+        <v>40.7554749</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>-73.9538405</v>
+        <v>-73.9779336</v>
       </c>
       <c r="L25" s="7" t="n">
         <v>100</v>
@@ -2017,17 +2017,17 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Midtown Dental Group Upper East Side</t>
+          <t>NYC Smile Spa</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>(212) 588-1809</t>
+          <t>(646) 374-2242</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>30 E 60th St Ste 2402, New York, NY 10022, USA</t>
+          <t>30 E 60th St Ste 1201, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -2037,25 +2037,25 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>https://midtowndentalgroup.com/locations/uppereastside/</t>
+          <t>https://www.nycsmilespa.com/</t>
         </is>
       </c>
       <c r="G26" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>505</v>
+        <v>395</v>
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: 8:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J26" s="9" t="n">
-        <v>40.763742</v>
+        <v>40.7637066</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>-73.97019589999999</v>
+        <v>-73.970242</v>
       </c>
       <c r="L26" s="9" t="n">
         <v>100</v>
@@ -2072,17 +2072,17 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Midtown Dental Group Fashion District</t>
+          <t>Soho Smile - Cosmetic Dentist NYC</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>(212) 730-4440</t>
+          <t>(212) 334-7330</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>241 W 37th St Ground Floor, New York, NY 10018, USA</t>
+          <t>206 Spring St 5th Floor, New York, NY 10012, USA</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -2092,25 +2092,25 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>http://www.midtowndentalgroup.com/</t>
+          <t>https://www.sohosmile.com/</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>734</v>
+        <v>210</v>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:45 PM</t>
+          <t>Monday: 9:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>40.7538706</v>
+        <v>40.7252587</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>-73.9909457</v>
+        <v>-74.0037653</v>
       </c>
       <c r="L27" s="7" t="n">
         <v>100</v>
@@ -2127,17 +2127,17 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Preferred Dental Care - Chelsea Dentist</t>
+          <t>TriBeCa Dental Associates | Murray</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>(212) 594-7171</t>
+          <t>(212) 671-3749</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>135 W 27th St, New York, NY 10001, USA</t>
+          <t>21 Murray St 4th floor, New York, NY 10007, USA</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2147,25 +2147,25 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>https://www.preferreddentalcare.com/locations/chelsea-ny-location</t>
+          <t>https://tribeca.dental/</t>
         </is>
       </c>
       <c r="G28" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>2341</v>
+        <v>1505</v>
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>Monday: 7:00 AM – 9:00 PM</t>
+          <t>Monday: 8:00 AM – 4:00 PM</t>
         </is>
       </c>
       <c r="J28" s="9" t="n">
-        <v>40.7462879</v>
+        <v>40.7137936</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>-73.9924206</v>
+        <v>-74.0081888</v>
       </c>
       <c r="L28" s="9" t="n">
         <v>100</v>
@@ -2182,17 +2182,17 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Dental House</t>
+          <t>Tribeca Dental Care</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>(212) 888-3384</t>
+          <t>(212) 431-4582</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>41 7th Ave, New York, NY 10011, USA</t>
+          <t>402 Broadway, New York, NY 10013, USA</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2202,25 +2202,25 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>http://www.dentalhousenyc.com/</t>
+          <t>https://tribecanydentistoffice.com/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gbp</t>
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>793</v>
+        <v>1164</v>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 10:00 AM – 6:30 PM</t>
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>40.7379183</v>
+        <v>40.7186949</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>-73.99990369999999</v>
+        <v>-74.0021775</v>
       </c>
       <c r="L29" s="7" t="n">
         <v>100</v>
@@ -2237,17 +2237,17 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Modern Dental of Manhattan</t>
+          <t>212 Dental Care</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>(212) 758-1000</t>
+          <t>(888) 506-9583</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>425 Madison Ave Rm 500, New York, NY 10017, USA</t>
+          <t>286 Madison Ave 10th Floor, New York, NY 10017, USA</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -2257,25 +2257,25 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>https://www.manhattandentists.com/</t>
+          <t>http://212dentalcare.com/</t>
         </is>
       </c>
       <c r="G30" s="9" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>235</v>
+        <v>3272</v>
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 8:00 PM</t>
         </is>
       </c>
       <c r="J30" s="9" t="n">
-        <v>40.7569869</v>
+        <v>40.751693</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>-73.975942</v>
+        <v>-73.9803106</v>
       </c>
       <c r="L30" s="9" t="n">
         <v>100</v>
@@ -2292,17 +2292,17 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Beautiful Smiles Dental Associates</t>
+          <t>Dental House</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>(516) 715-5650</t>
+          <t>(212) 888-3384</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>2 W 46th St Ste 1003 10th Floor, New York, NY 10036, USA</t>
+          <t>41 7th Ave, New York, NY 10011, USA</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2312,25 +2312,25 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>https://www.beautifulsmilesdentalassociates.com/</t>
+          <t>http://www.dentalhousenyc.com/</t>
         </is>
       </c>
       <c r="G31" s="7" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>815</v>
+        <v>796</v>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>Monday: 8:30 AM – 6:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J31" s="7" t="n">
-        <v>40.756096</v>
+        <v>40.7379183</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>-73.9798129</v>
+        <v>-73.99990369999999</v>
       </c>
       <c r="L31" s="7" t="n">
         <v>100</v>
@@ -2347,17 +2347,17 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>The Exchange Dental Group</t>
+          <t>Preferred Dental Care - Chelsea Dentist</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>(646) 780-5410</t>
+          <t>(212) 594-7171</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>39 Broadway Rm 2115, New York, NY 10006, USA</t>
+          <t>135 W 27th St, New York, NY 10001, USA</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -2367,25 +2367,25 @@
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>https://www.theexchangedentalgroup.com/</t>
+          <t>https://www.preferreddentalcare.com/locations/chelsea-ny-location</t>
         </is>
       </c>
       <c r="G32" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>1249</v>
+        <v>2346</v>
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 7:00 PM</t>
+          <t>Monday: 7:00 AM – 9:00 PM</t>
         </is>
       </c>
       <c r="J32" s="9" t="n">
-        <v>40.7063221</v>
+        <v>40.7462879</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>-74.01333289999999</v>
+        <v>-73.9924206</v>
       </c>
       <c r="L32" s="9" t="n">
         <v>100</v>
@@ -2402,17 +2402,17 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Manhattan Bridge Orthodontics</t>
+          <t>Dentist on Madison</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>(212) 274-0477</t>
+          <t>(212) 227-4600</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>77 Bowery 6th Floor, New York, NY 10002, USA</t>
+          <t>274 Madison Ave Rm 202, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2422,25 +2422,25 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>https://www.manhattanbridgeortho.com/</t>
+          <t>http://dentistonmadison.com/?utm_campaign=gmb</t>
         </is>
       </c>
       <c r="G33" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>1514</v>
+        <v>388</v>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 7:00 PM</t>
+          <t>Monday: 12:00 – 8:00 PM</t>
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>40.71666949999999</v>
+        <v>40.7514023</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>-73.99553539999999</v>
+        <v>-73.980757</v>
       </c>
       <c r="L33" s="7" t="n">
         <v>100</v>
@@ -2457,17 +2457,17 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>iSmile Orthodontics - NYC</t>
+          <t>Manhattan Bridge Orthodontics</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>(646) 863-2181</t>
+          <t>(212) 274-0477</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>4779 Broadway, New York, NY 10034, USA</t>
+          <t>77 Bowery 6th Floor, New York, NY 10002, USA</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
@@ -2477,25 +2477,25 @@
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>https://ismileorthodontics.com/inwood/</t>
+          <t>https://www.manhattanbridgeortho.com/</t>
         </is>
       </c>
       <c r="G34" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>1006</v>
+        <v>1517</v>
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 10:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J34" s="9" t="n">
-        <v>40.8659992</v>
+        <v>40.71666949999999</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>-73.92655979999999</v>
+        <v>-73.99553539999999</v>
       </c>
       <c r="L34" s="9" t="n">
         <v>100</v>
@@ -2512,17 +2512,17 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>NYC Orthodontics</t>
+          <t>iSmile Orthodontics - NYC</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>(212) 245-5121</t>
+          <t>(646) 863-2181</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>30 Central Park S RM 2A, New York, NY 10019, USA</t>
+          <t>4779 Broadway, New York, NY 10034, USA</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -2532,28 +2532,28 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>https://www.orthonyc.com/</t>
+          <t>https://ismileorthodontics.com/inwood/</t>
         </is>
       </c>
       <c r="G35" s="7" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>54</v>
+        <v>1006</v>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>Monday: 12:00 – 6:30 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J35" s="7" t="n">
-        <v>40.7649517</v>
+        <v>40.8659992</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>-73.9750827</v>
+        <v>-73.92655979999999</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="M35" s="8" t="inlineStr">
         <is>
@@ -2567,17 +2567,17 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Manhattan EastSide Orthodontics</t>
+          <t>NYC Orthodontics</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>(212) 289-8989</t>
+          <t>(212) 245-5121</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>207 E 94th St #501, New York, NY 10128, USA</t>
+          <t>30 Central Park S RM 2A, New York, NY 10019, USA</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -2587,28 +2587,28 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>https://manhattaneastsideorthodontics.com/</t>
+          <t>https://www.orthonyc.com/</t>
         </is>
       </c>
       <c r="G36" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>429</v>
+        <v>57</v>
       </c>
       <c r="I36" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: 12:00 – 6:30 PM</t>
         </is>
       </c>
       <c r="J36" s="9" t="n">
-        <v>40.783778</v>
+        <v>40.7649517</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>-73.949438</v>
+        <v>-73.9750827</v>
       </c>
       <c r="L36" s="9" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="M36" s="8" t="inlineStr">
         <is>
@@ -2622,17 +2622,17 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Brite Orthodontics - Harlem (Central Park North Orthodontics)</t>
+          <t>Manhattan EastSide Orthodontics</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>(212) 866-9800</t>
+          <t>(212) 289-8989</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>1851 Adam Clayton Powell Jr Blvd, New York, NY 10026, USA</t>
+          <t>207 E 94th St #501, New York, NY 10128, USA</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -2642,14 +2642,14 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>https://www.briteorthodontics.com/locations/newyork-ny/</t>
+          <t>https://manhattaneastsideorthodontics.com/</t>
         </is>
       </c>
       <c r="G37" s="7" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>673</v>
+        <v>429</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
@@ -2657,10 +2657,10 @@
         </is>
       </c>
       <c r="J37" s="7" t="n">
-        <v>40.8009348</v>
+        <v>40.783778</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>-73.95373900000001</v>
+        <v>-73.949438</v>
       </c>
       <c r="L37" s="7" t="n">
         <v>100</v>
@@ -2677,17 +2677,17 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Goodman Orthodontics</t>
+          <t>Brite Orthodontics - Harlem (Central Park North Orthodontics)</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>(212) 688-4663</t>
+          <t>(212) 866-9800</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>440 E 57th St B, New York, NY 10022, USA</t>
+          <t>1851 Adam Clayton Powell Jr Blvd, New York, NY 10026, USA</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -2697,25 +2697,25 @@
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>http://www.goodortho.com/</t>
+          <t>https://www.briteorthodontics.com/locations/newyork-ny/</t>
         </is>
       </c>
       <c r="G38" s="9" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>275</v>
+        <v>673</v>
       </c>
       <c r="I38" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 4:00 PM</t>
+          <t>Monday: 9:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J38" s="9" t="n">
-        <v>40.7575229</v>
+        <v>40.8009348</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>-73.9616418</v>
+        <v>-73.95373900000001</v>
       </c>
       <c r="L38" s="9" t="n">
         <v>100</v>
@@ -2732,17 +2732,17 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Gramercy Orthodontics</t>
+          <t>Smile Pop - Dr. Courtney Barry Orthodontist</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>(212) 777-9177</t>
+          <t>(646) 770-2091</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>200 E 15th St STE PRB, New York, NY 10003, USA</t>
+          <t>76 Madison Ave, New York, NY 10016, USA</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2752,28 +2752,28 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>https://gramercyorthonyc.com/</t>
+          <t>http://www.smilepop.com/</t>
         </is>
       </c>
       <c r="G39" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>161</v>
+        <v>445</v>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 7:00 PM</t>
+          <t>Monday: 10:00 AM – 4:00 PM</t>
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>40.7337844</v>
+        <v>40.74397099999999</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>-73.98647919999999</v>
+        <v>-73.9860561</v>
       </c>
       <c r="L39" s="7" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M39" s="8" t="inlineStr">
         <is>
@@ -2787,17 +2787,17 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Bronsky Orthodontics</t>
+          <t>Fellow Orthodontist</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>(212) 758-0040</t>
+          <t>(917) 451-2999</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>530 Park Ave APT 1G, New York, NY 10065, USA</t>
+          <t>49 E 18th St, New York, NY 10003, USA</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
@@ -2807,25 +2807,25 @@
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>http://www.bronskyorthodontics.com/?utm_source=GMBlisting&amp;utm_medium=organic</t>
+          <t>https://felloworthodontist.com/</t>
         </is>
       </c>
       <c r="G40" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>481</v>
+        <v>234</v>
       </c>
       <c r="I40" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 5:00 PM</t>
+          <t>Monday: 10:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J40" s="9" t="n">
-        <v>40.7641462</v>
+        <v>40.7375877</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>-73.96946849999999</v>
+        <v>-73.98918399999999</v>
       </c>
       <c r="L40" s="9" t="n">
         <v>100</v>
@@ -2842,17 +2842,17 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Smile Pop - Dr. Courtney Barry Orthodontist</t>
+          <t>Bronsky Orthodontics</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>(646) 770-2091</t>
+          <t>(212) 758-0040</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>76 Madison Ave, New York, NY 10016, USA</t>
+          <t>530 Park Ave APT 1G, New York, NY 10065, USA</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2862,25 +2862,25 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>http://www.smilepop.com/</t>
+          <t>http://www.bronskyorthodontics.com/?utm_source=GMBlisting&amp;utm_medium=organic</t>
         </is>
       </c>
       <c r="G41" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>444</v>
+        <v>481</v>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 4:00 PM</t>
+          <t>Monday: 8:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>40.74397099999999</v>
+        <v>40.7641462</v>
       </c>
       <c r="K41" s="7" t="n">
-        <v>-73.9860561</v>
+        <v>-73.96946849999999</v>
       </c>
       <c r="L41" s="7" t="n">
         <v>100</v>
@@ -2897,17 +2897,17 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Salzer Orthodontics, Dr. Jennifer Salzer</t>
+          <t>Goodman Orthodontics</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>(212) 755-2333</t>
+          <t>(212) 688-4663</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>553 Park Ave, New York, NY 10065, USA</t>
+          <t>440 E 57th St B, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
@@ -2917,28 +2917,28 @@
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>https://lsortho.com/contact-orthodontist-nyc</t>
+          <t>http://www.goodortho.com/</t>
         </is>
       </c>
       <c r="G42" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>177</v>
+        <v>275</v>
       </c>
       <c r="I42" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 8:00 AM – 4:00 PM</t>
         </is>
       </c>
       <c r="J42" s="9" t="n">
-        <v>40.7645406</v>
+        <v>40.7575229</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>-73.9683215</v>
+        <v>-73.9616418</v>
       </c>
       <c r="L42" s="9" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
@@ -2952,48 +2952,48 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Jackson Heights Orthodontics</t>
+          <t>Gramercy Orthodontics</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>(718) 335-4444</t>
+          <t>(212) 777-9177</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>37-43 77th St, Jackson Heights, NY 11372, USA</t>
+          <t>200 E 15th St STE PRB, New York, NY 10003, USA</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Jackson Heights</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>http://jhoortho.com/</t>
+          <t>https://gramercyorthonyc.com/</t>
         </is>
       </c>
       <c r="G43" s="7" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>1337</v>
+        <v>163</v>
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: 10:00 AM – 7:00 PM</t>
         </is>
       </c>
       <c r="J43" s="7" t="n">
-        <v>40.7479692</v>
+        <v>40.7337844</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>-73.88860989999999</v>
+        <v>-73.98647919999999</v>
       </c>
       <c r="L43" s="7" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
@@ -3007,17 +3007,17 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Wall Street Orthodontics</t>
+          <t>House of Orthodontia - Manhattan</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>(212) 871-9835</t>
+          <t>(212) 392-4789</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>111 Broadway APT 1707, New York, NY 10006, USA</t>
+          <t>601 E 12th St, New York, NY 10009, USA</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -3027,28 +3027,28 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>http://wallstreetortho.com/</t>
+          <t>https://houseoforthodontia.com/</t>
         </is>
       </c>
       <c r="G44" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: Closed</t>
         </is>
       </c>
       <c r="J44" s="9" t="n">
-        <v>40.7086853</v>
+        <v>40.7281888</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>-74.01154869999999</v>
+        <v>-73.9788071</v>
       </c>
       <c r="L44" s="9" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
@@ -3062,17 +3062,17 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Straight Set Orthodontics | Harlem</t>
+          <t>Manhattan Family Orthodontics-Uptown</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>(212) 996-7300</t>
+          <t>(347) 767-5668</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>241 Malcolm X Blvd, New York, NY 10027, USA</t>
+          <t>207 E 63rd St, New York, NY 10022, USA</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -3082,28 +3082,28 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>https://www.straightsetortho.com/harlem</t>
+          <t>https://www.manhattanfamilyorthodontics.com/</t>
         </is>
       </c>
       <c r="G45" s="7" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>677</v>
+        <v>160</v>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 1:00 – 6:00 PM</t>
         </is>
       </c>
       <c r="J45" s="7" t="n">
-        <v>40.8060963</v>
+        <v>40.7640232</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>-73.94716439999999</v>
+        <v>-73.96417579999999</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
@@ -3117,45 +3117,45 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Fellow Orthodontist</t>
+          <t>Jackson Heights Orthodontics</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>(917) 451-2999</t>
+          <t>(718) 335-4444</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>49 E 18th St, New York, NY 10003, USA</t>
+          <t>37-43 77th St, Jackson Heights, NY 11372, USA</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Jackson Heights</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>https://felloworthodontist.com/</t>
+          <t>http://jhoortho.com/</t>
         </is>
       </c>
       <c r="G46" s="9" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>234</v>
+        <v>1336</v>
       </c>
       <c r="I46" s="9" t="inlineStr">
         <is>
-          <t>Monday: 10:00 AM – 5:00 PM</t>
+          <t>Monday: 9:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J46" s="9" t="n">
-        <v>40.7375877</v>
+        <v>40.7479692</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>-73.98918399999999</v>
+        <v>-73.88860989999999</v>
       </c>
       <c r="L46" s="9" t="n">
         <v>100</v>
@@ -3172,17 +3172,17 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Central Park Orthodontics</t>
+          <t>Wall Street Orthodontics</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>(212) 362-4400</t>
+          <t>(212) 871-9835</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>271A Central Park West, (entrance on, W 87th St, New York, NY 10024, USA</t>
+          <t>111 Broadway APT 1707, New York, NY 10006, USA</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -3192,25 +3192,25 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>https://www.centralparkorthodontics.com/</t>
+          <t>http://wallstreetortho.com/</t>
         </is>
       </c>
       <c r="G47" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 9:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J47" s="7" t="n">
-        <v>40.786237</v>
+        <v>40.7086853</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>-73.969014</v>
+        <v>-74.01154869999999</v>
       </c>
       <c r="L47" s="7" t="n">
         <v>77</v>
@@ -3227,17 +3227,17 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Gibbs Orthodontic Associates, P.C : Invisalign, Braces and Dentofacial Orthopedics</t>
+          <t>Straight Set Orthodontics | Harlem</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>(212) 535-4111</t>
+          <t>(212) 996-7300</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>40 E 84th St, New York, NY 10028, USA</t>
+          <t>241 Malcolm X Blvd, New York, NY 10027, USA</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -3247,28 +3247,28 @@
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>https://www.gibbsortho.com/</t>
+          <t>https://www.straightsetortho.com/harlem</t>
         </is>
       </c>
       <c r="G48" s="9" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>186</v>
+        <v>678</v>
       </c>
       <c r="I48" s="9" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 5:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J48" s="9" t="n">
-        <v>40.7793093</v>
+        <v>40.8060963</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>-73.95947029999999</v>
+        <v>-73.94716439999999</v>
       </c>
       <c r="L48" s="9" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M48" s="8" t="inlineStr">
         <is>
@@ -3282,17 +3282,17 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Orthodontics Center of NYC</t>
+          <t>Central Park West Orthodontics</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>(646) 491-7133</t>
+          <t>(917) 336-8548</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>263 West End Ave Fl 1, New York, NY 10023, USA</t>
+          <t>327 Central Prk W #1a, New York, NY 10025, USA</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -3302,32 +3302,32 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>https://www.orthodonticscenternyc.com/</t>
+          <t>https://cpworthodontic.com/?utm_source=google.com&amp;utm_medium=business+profile</t>
         </is>
       </c>
       <c r="G49" s="7" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>12</v>
+        <v>135</v>
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>Monday: 9:00 AM – 6:00 PM</t>
+          <t>Monday: 10:00 AM – 5:00 PM</t>
         </is>
       </c>
       <c r="J49" s="7" t="n">
-        <v>40.7800807</v>
+        <v>40.7897119</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>-73.9845136</v>
+        <v>-73.96653289999999</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="M49" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>93</v>
+      </c>
+      <c r="M49" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Lemchen Salzer Orthodontics</t>
+          <t>Salzer Orthodontics, Dr. Jennifer Salzer</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -3357,14 +3357,14 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>http://www.lsortho.com/</t>
+          <t>https://lsortho.com/contact-orthodontist-nyc</t>
         </is>
       </c>
       <c r="G50" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>313</v>
+        <v>177</v>
       </c>
       <c r="I50" s="9" t="inlineStr">
         <is>
@@ -3372,13 +3372,13 @@
         </is>
       </c>
       <c r="J50" s="9" t="n">
-        <v>40.76448</v>
+        <v>40.7645406</v>
       </c>
       <c r="K50" s="9" t="n">
-        <v>-73.96826279999999</v>
+        <v>-73.9683215</v>
       </c>
       <c r="L50" s="9" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M50" s="8" t="inlineStr">
         <is>
@@ -3392,17 +3392,17 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Manhattan Family Orthodontics-Uptown</t>
+          <t>Upper Eastside Orthodontists</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>(347) 767-5668</t>
+          <t>(212) 360-0835</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>207 E 63rd St, New York, NY 10022, USA</t>
+          <t>153 E 87th St APT 1B, New York, NY 10128, USA</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -3412,28 +3412,28 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>https://www.manhattanfamilyorthodontics.com/</t>
+          <t>https://www.ueso.org/?utm_source=local_directory&amp;utm_medium=referral&amp;utm_campaign=directory-listing</t>
         </is>
       </c>
       <c r="G51" s="7" t="n">
         <v>4.9</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>159</v>
+        <v>476</v>
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Monday: 1:00 – 6:00 PM</t>
+          <t>Monday: Closed</t>
         </is>
       </c>
       <c r="J51" s="7" t="n">
-        <v>40.7640232</v>
+        <v>40.7802182</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>-73.96417579999999</v>
+        <v>-73.9546495</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M51" s="8" t="inlineStr">
         <is>
@@ -3447,17 +3447,17 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Mid-Manhattan Oral Surgery, PC</t>
+          <t>Central Park Orthodontics</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>(212) 918-1859</t>
+          <t>(212) 362-4400</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>36 West 44th Street, Suite 600 Between, 5th and 6th Avenue, New York, NY 10036, USA</t>
+          <t>271A Central Park West, (entrance on, W 87th St, New York, NY 10024, USA</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -3467,28 +3467,28 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>https://www.midmanhattanoralsurgery.com/</t>
+          <t>https://www.centralparkorthodontics.com/</t>
         </is>
       </c>
       <c r="G52" s="9" t="n">
         <v>4.9</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>895</v>
+        <v>60</v>
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
-          <t>Monday: 8:00 AM – 5:00 PM</t>
+          <t>Monday: 9:00 AM – 6:00 PM</t>
         </is>
       </c>
       <c r="J52" s="9" t="n">
-        <v>40.7555517</v>
+        <v>40.786237</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>-73.9819631</v>
+        <v>-73.969014</v>
       </c>
       <c r="L52" s="9" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="M52" s="8" t="inlineStr">
         <is>

</xml_diff>